<commit_message>
feat: add DOCX and XLSX task packages
</commit_message>
<xml_diff>
--- a/tasks/xlsx/cowork-bench-sf-regional-sales-forecast/solution/Sales_Forecast.xlsx
+++ b/tasks/xlsx/cowork-bench-sf-regional-sales-forecast/solution/Sales_Forecast.xlsx
@@ -10,16 +10,26 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historical'!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Forecast'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Forecast Notes'!$A$1:$B$6</definedName>
+  </definedNames>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +37,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017365D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +68,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -124,6 +153,56 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Historical_Sales" displayName="Historical_Sales" ref="A1:D16" headerRowCount="1">
+  <autoFilter ref="A1:D16"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Region"/>
+    <tableColumn id="2" name="Month"/>
+    <tableColumn id="3" name="Orders"/>
+    <tableColumn id="4" name="Revenue"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Regional_Forecast" displayName="Regional_Forecast" ref="A1:F6" headerRowCount="1">
+  <autoFilter ref="A1:F6"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Region"/>
+    <tableColumn id="2" name="Trailing_3M_Avg"/>
+    <tableColumn id="3" name="GDP_Growth_Pct"/>
+    <tableColumn id="4" name="Economic_Adjustment"/>
+    <tableColumn id="5" name="Adjusted_Monthly_Forecast"/>
+    <tableColumn id="6" name="Next_Quarter_Forecast"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Forecast_Summary" displayName="Forecast_Summary" ref="A1:B11" headerRowCount="1">
+  <autoFilter ref="A1:B11"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Metric"/>
+    <tableColumn id="2" name="Value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Forecast_Notes" displayName="Forecast_Notes" ref="A1:B6" headerRowCount="1">
+  <autoFilter ref="A1:B6"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Раздел"/>
+    <tableColumn id="2" name="Содержание"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -417,24 +496,30 @@
   </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
@@ -454,7 +539,7 @@
       <c r="C2" t="n">
         <v>159</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>22569.49</v>
       </c>
     </row>
@@ -472,7 +557,7 @@
       <c r="C3" t="n">
         <v>198</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>33440.58</v>
       </c>
     </row>
@@ -490,7 +575,7 @@
       <c r="C4" t="n">
         <v>196</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>34541.01</v>
       </c>
     </row>
@@ -508,7 +593,7 @@
       <c r="C5" t="n">
         <v>169</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>30465.15</v>
       </c>
     </row>
@@ -526,7 +611,7 @@
       <c r="C6" t="n">
         <v>161</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>20983.26</v>
       </c>
     </row>
@@ -544,7 +629,7 @@
       <c r="C7" t="n">
         <v>161</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>21174.11</v>
       </c>
     </row>
@@ -562,7 +647,7 @@
       <c r="C8" t="n">
         <v>164</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>21112.39</v>
       </c>
     </row>
@@ -580,7 +665,7 @@
       <c r="C9" t="n">
         <v>157</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>23321.96</v>
       </c>
     </row>
@@ -598,7 +683,7 @@
       <c r="C10" t="n">
         <v>168</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>31243.81</v>
       </c>
     </row>
@@ -616,7 +701,7 @@
       <c r="C11" t="n">
         <v>169</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>30899.91</v>
       </c>
     </row>
@@ -634,7 +719,7 @@
       <c r="C12" t="n">
         <v>152</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>20088.71</v>
       </c>
     </row>
@@ -652,7 +737,7 @@
       <c r="C13" t="n">
         <v>167</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>23103.02</v>
       </c>
     </row>
@@ -670,7 +755,7 @@
       <c r="C14" t="n">
         <v>162</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
         <v>29207.02</v>
       </c>
     </row>
@@ -688,7 +773,7 @@
       <c r="C15" t="n">
         <v>184</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="2" t="n">
         <v>23384.92</v>
       </c>
     </row>
@@ -706,12 +791,16 @@
       <c r="C16" t="n">
         <v>171</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="2" t="n">
         <v>28117.89</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -723,34 +812,42 @@
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Trailing_3M_Avg</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>GDP_Growth_Pct</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Economic_Adjustment</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Adjusted_Monthly_Forecast</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Next_Quarter_Forecast</t>
         </is>
@@ -762,19 +859,19 @@
           <t>Азиатско-Тихоокеанский регион</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>30183.69</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>3.8</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="4" t="n">
         <v>1.038</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>31330.67</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>93992.00999999999</v>
       </c>
     </row>
@@ -784,19 +881,19 @@
           <t>Европа</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>24207.51</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="4" t="n">
         <v>1.015</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>24570.62</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>73711.86</v>
       </c>
     </row>
@@ -806,19 +903,19 @@
           <t>Латинская Америка</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>25226.05</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="4" t="n">
         <v>1.012</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>25528.76</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>76586.28</v>
       </c>
     </row>
@@ -828,19 +925,19 @@
           <t>Ближний Восток</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>24697.21</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="4" t="n">
         <v>1.025</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>25314.64</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>75943.92</v>
       </c>
     </row>
@@ -850,24 +947,28 @@
           <t>Северная Америка</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>26903.28</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="3" t="n">
         <v>2.1</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="4" t="n">
         <v>1.021</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>27468.25</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>82404.75</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -879,14 +980,18 @@
   </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -898,7 +1003,7 @@
           <t>Total_Q4_2025_Revenue</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>393653.23</v>
       </c>
     </row>
@@ -908,7 +1013,7 @@
           <t>Total_Monthly_Average</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>131217.74</v>
       </c>
     </row>
@@ -918,7 +1023,7 @@
           <t>Total_Q1_2026_Forecast</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>402638.85</v>
       </c>
     </row>
@@ -928,7 +1033,7 @@
           <t>QoQ_Growth_Pct</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>2.3</v>
       </c>
     </row>
@@ -950,7 +1055,7 @@
           <t>Highest_Forecast_Amount</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="2" t="n">
         <v>93992.02</v>
       </c>
     </row>
@@ -972,7 +1077,7 @@
           <t>Lowest_Forecast_Amount</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="2" t="n">
         <v>73711.86</v>
       </c>
     </row>
@@ -994,11 +1099,109 @@
           <t>Regions_Count</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="3" t="n">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Содержание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Краткое резюме</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Прогноз выручки на I квартал 2026 года: $402,638.85; IV квартал 2025 года: $393,653.23; рост: 2.3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Для каждого региона: средняя выручка за октябрь-декабрь 2025 × (1 + рост ВВП / 100); квартальный прогноз равен трём месячным.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Региональный анализ</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Азиатско-Тихоокеанский регион: $93,992.01, ВВП 3.8%; Европа: $73,711.86, ВВП 1.5%; Латинская Америка: $76,586.28, ВВП 1.2%; Ближний Восток: $75,943.92, ВВП 2.5%; Северная Америка: $82,404.75, ВВП 2.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Ключевые допущения</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Предполагаются стабильные цены, продуктовый портфель, охват команды продаж и экономические условия; новые промоакции и рыночные шоки не моделируются.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Рекомендации</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Усилить коммерческий фокус на Азиатско-Тихоокеанский регион; для Европы использовать целевые кампании и ежемесячно сверять прогноз с фактом.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>